<commit_message>
docs: completa las politicas de direccion y corrige las referencias rotas de C-Direccion
</commit_message>
<xml_diff>
--- a/docs/MuestreoDatosModeloDominio_Imexcol_Oct29.xlsx
+++ b/docs/MuestreoDatosModeloDominio_Imexcol_Oct29.xlsx
@@ -81,7 +81,7 @@
     <sheet name="E-EnvioRastreo" sheetId="51" r:id="rId66"/>
     <sheet name="P-EnvioRastreo " sheetId="66" r:id="rId67"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -13137,7 +13137,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:Z37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
@@ -13806,7 +13806,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1">
+    <row r="19" spans="1:11" ht="62" customHeight="1">
       <c r="A19" s="252"/>
       <c r="B19" s="252"/>
       <c r="C19" s="252"/>
@@ -13829,7 +13829,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1">
+    <row r="20" spans="1:11" ht="62" customHeight="1">
       <c r="A20" s="253"/>
       <c r="B20" s="253"/>
       <c r="C20" s="253"/>
@@ -13837,10 +13837,22 @@
       <c r="E20" s="253"/>
       <c r="F20" s="253"/>
       <c r="G20" s="253"/>
-      <c r="H20" s="253"/>
-      <c r="I20" s="253"/>
-      <c r="J20" s="253"/>
-      <c r="K20" s="253"/>
+      <c r="H20" s="251" t="str">
+        <f>'E-Direccion'!G9</f>
+        <v>DIR-POL-03</v>
+      </c>
+      <c r="I20" s="262" t="str">
+        <f>'E-Direccion'!H9</f>
+        <v>Un cliente no puede registrar dos direcciones con la misma combinación de calle, ciudad, departamento </v>
+      </c>
+      <c r="J20" s="251" t="inlineStr">
+        <is>
+          <t>Generar excepción indicando que el cliente ya tiene registrada una dirección con la misma calle, ciudad y departamento.</t>
+        </is>
+      </c>
+      <c r="K20" s="251" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="77.25" customHeight="1">
       <c r="A21" s="190" t="str">
@@ -13881,108 +13893,134 @@
         <v>141</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="57.75" customHeight="1">
-      <c r="A22" s="254" t="str">
-        <f>'E-Direccion'!B11</f>
+    <row r="22" spans="1:13" ht="100" customHeight="1">
+      <c r="A22" s="190"/>
+      <c r="B22" s="190"/>
+      <c r="C22" s="190"/>
+      <c r="D22" s="190"/>
+      <c r="E22" s="190"/>
+      <c r="F22" s="190"/>
+      <c r="G22" s="190"/>
+      <c r="H22" s="190" t="str">
+        <f>'E-Direccion'!G11</f>
+        <v>DIR-POL-08</v>
+      </c>
+      <c r="I22" s="190" t="str">
+        <f>'E-Direccion'!H11</f>
+        <v>Una dirección asociada a pedidos en curso (Pendiente, Confirmado, Preparando o Enviado) no se puede modificar.</v>
+      </c>
+      <c r="J22" s="190" t="inlineStr">
+        <is>
+          <t>Generar excepción indicando que la dirección está bloqueada temporalmente porque tiene pedidos en curso.</t>
+        </is>
+      </c>
+      <c r="K22" s="190" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="57.75" customHeight="1">
+      <c r="A23" s="254" t="str">
+        <f>'E-Direccion'!B12</f>
         <v>Eliminar dirección</v>
       </c>
-      <c r="B22" s="254" t="str">
-        <f>'E-Direccion'!C11</f>
+      <c r="B23" s="254" t="str">
+        <f>'E-Direccion'!C12</f>
         <v xml:space="preserve">	Quitar una dirección de la libreta de direcciones del usuario para que no aparezca en futuras compras. </v>
       </c>
-      <c r="C22" s="260" t="s">
+      <c r="C23" s="260" t="s">
         <v>368</v>
       </c>
-      <c r="D22" s="260" t="s">
+      <c r="D23" s="260" t="s">
         <v>244</v>
       </c>
-      <c r="E22" s="260" t="s">
+      <c r="E23" s="260" t="s">
         <v>369</v>
       </c>
-      <c r="F22" s="260" t="s">
+      <c r="F23" s="260" t="s">
         <v>138</v>
       </c>
-      <c r="G22" s="260" t="s">
+      <c r="G23" s="260" t="s">
         <v>370</v>
       </c>
-      <c r="H22" s="185" t="str">
-        <f>'E-Direccion'!G11</f>
+      <c r="H23" s="185" t="str">
+        <f>'E-Direccion'!G12</f>
         <v>DIR-POL-05</v>
       </c>
-      <c r="I22" s="185" t="str">
-        <f>'E-Direccion'!H11</f>
+      <c r="I23" s="185" t="str">
+        <f>'E-Direccion'!H12</f>
         <v>El idDireccion a eliminar debe existir previamente en el sistema</v>
       </c>
-      <c r="J22" s="185" t="s">
+      <c r="J23" s="185" t="s">
         <v>371</v>
-      </c>
-      <c r="K22" s="185" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="87" customHeight="1">
-      <c r="A23" s="253"/>
-      <c r="B23" s="253"/>
-      <c r="C23" s="253"/>
-      <c r="D23" s="253"/>
-      <c r="E23" s="253"/>
-      <c r="F23" s="253"/>
-      <c r="G23" s="253"/>
-      <c r="H23" s="185" t="e">
-        <f>'E-Direccion'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I23" s="185">
-        <f>'E-Direccion'!H12</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="185" t="s">
-        <v>372</v>
       </c>
       <c r="K23" s="185" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="87" customHeight="1">
-      <c r="A24" s="191">
-        <f>'E-Direccion'!B13</f>
-        <v>0</v>
-      </c>
-      <c r="B24" s="191" t="str">
-        <f>'E-Direccion'!C11</f>
-        <v xml:space="preserve">	Quitar una dirección de la libreta de direcciones del usuario para que no aparezca en futuras compras. </v>
-      </c>
-      <c r="C24" s="186" t="s">
+      <c r="A24" s="253"/>
+      <c r="B24" s="253"/>
+      <c r="C24" s="253"/>
+      <c r="D24" s="253"/>
+      <c r="E24" s="253"/>
+      <c r="F24" s="253"/>
+      <c r="G24" s="253"/>
+      <c r="H24" s="185" t="str">
+        <f>'E-Direccion'!G13</f>
+        <v>DIR-POL-06</v>
+      </c>
+      <c r="I24" s="185" t="str">
+        <f>'E-Direccion'!H13</f>
+        <v>Una dirección asociada a pedidos no se puede eliminar; el cliente puede registrar una nueva.</v>
+      </c>
+      <c r="J24" s="185" t="inlineStr">
+        <is>
+          <t>Generar excepción indicando que la dirección no se puede eliminar porque está asociada a pedidos.</t>
+        </is>
+      </c>
+      <c r="K24" s="185" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="87" customHeight="1">
+      <c r="A25" s="191" t="str">
+        <f>'E-Direccion'!B14</f>
+        <v>Consultar direcciones</v>
+      </c>
+      <c r="B25" s="191" t="str">
+        <f>'E-Direccion'!C14</f>
+        <v>Listar las direcciones registradas por el cliente para seleccionarlas en el checkout.</v>
+      </c>
+      <c r="C25" s="186" t="s">
         <v>373</v>
       </c>
-      <c r="D24" s="181" t="s">
+      <c r="D25" s="181" t="s">
         <v>244</v>
       </c>
-      <c r="E24" s="181" t="s">
+      <c r="E25" s="181" t="s">
         <v>374</v>
       </c>
-      <c r="F24" s="181" t="s">
+      <c r="F25" s="181" t="s">
         <v>375</v>
       </c>
-      <c r="G24" s="182" t="s">
+      <c r="G25" s="182" t="s">
         <v>376</v>
       </c>
-      <c r="H24" s="181">
-        <f>'E-Direccion'!G13</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="181">
-        <f>'E-Direccion'!H13</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="183" t="s">
+      <c r="H25" s="181" t="str">
+        <f>'E-Direccion'!G14</f>
+        <v>DIR-POL-07</v>
+      </c>
+      <c r="I25" s="181" t="str">
+        <f>'E-Direccion'!H14</f>
+        <v>El cliente solo puede consultar sus propias direcciones; el administrador puede consultar todas.</v>
+      </c>
+      <c r="J25" s="183" t="s">
         <v>377</v>
       </c>
-      <c r="K24" s="183" t="s">
+      <c r="K25" s="183" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1"/>
     <row r="26" spans="1:11" ht="15.75" customHeight="1"/>
     <row r="27" spans="1:11" ht="15.75" customHeight="1"/>
     <row r="28" spans="1:11" ht="15.75" customHeight="1"/>
@@ -13990,38 +14028,42 @@
     <row r="30" spans="1:11" ht="15.75" customHeight="1"/>
     <row r="31" spans="1:11" ht="15.75" customHeight="1"/>
     <row r="32" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="31">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D18:D20"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="F23:F24"/>
     <mergeCell ref="C18:C20"/>
-    <mergeCell ref="H19:H20"/>
     <mergeCell ref="E18:E20"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="A23:A24"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="J16:K16"/>
-    <mergeCell ref="I19:I20"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="K19:K20"/>
     <mergeCell ref="B18:B20"/>
-    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="G23:G24"/>
     <mergeCell ref="F18:F20"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="E23:E24"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="B16:B17"/>
-    <mergeCell ref="J19:J20"/>
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de dominio'!A1" display="&lt;&lt; Ir al modelo de dominio" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
@@ -14043,7 +14085,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.5" style="62" customWidth="1"/>
@@ -14307,94 +14349,163 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A11" s="313" t="s">
+      <c r="A11" s="246"/>
+      <c r="B11" s="246"/>
+      <c r="C11" s="246"/>
+      <c r="D11" s="246"/>
+      <c r="E11" s="246"/>
+      <c r="F11" s="246"/>
+      <c r="G11" s="246" t="inlineStr">
+        <is>
+          <t>DIR-POL-08</t>
+        </is>
+      </c>
+      <c r="H11" s="246" t="inlineStr">
+        <is>
+          <t>Una dirección asociada a pedidos en curso (Pendiente, Confirmado, Preparando o Enviado) no se puede modificar.</t>
+        </is>
+      </c>
+      <c r="I11" s="246"/>
+      <c r="J11" s="246"/>
+      <c r="K11" s="246"/>
+    </row>
+    <row r="12" spans="1:13" ht="65.25" customHeight="1">
+      <c r="A12" s="313" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="313" t="s">
+      <c r="B12" s="313" t="s">
         <v>399</v>
       </c>
-      <c r="C11" s="313" t="s">
+      <c r="C12" s="313" t="s">
         <v>400</v>
       </c>
-      <c r="D11" s="313" t="str">
+      <c r="D12" s="313" t="str">
         <f>ListadoObjetosDominio!B5</f>
         <v>Dirección</v>
       </c>
-      <c r="E11" s="313" t="s">
+      <c r="E12" s="313" t="s">
         <v>368</v>
       </c>
-      <c r="F11" s="313" t="s">
+      <c r="F12" s="313" t="s">
         <v>401</v>
       </c>
-      <c r="G11" s="313" t="s">
+      <c r="G12" s="313" t="s">
         <v>402</v>
       </c>
-      <c r="H11" s="313" t="s">
+      <c r="H12" s="313" t="s">
         <v>403</v>
       </c>
-      <c r="I11" s="313" t="s">
+      <c r="I12" s="313" t="s">
         <v>180</v>
       </c>
-      <c r="J11" s="313" t="s">
+      <c r="J12" s="313" t="s">
         <v>404</v>
       </c>
-      <c r="K11" s="313" t="s">
+      <c r="K12" s="313" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A12" s="314"/>
-      <c r="B12" s="314"/>
-      <c r="C12" s="314"/>
-      <c r="D12" s="314"/>
-      <c r="E12" s="314"/>
-      <c r="F12" s="314"/>
-      <c r="G12" s="313"/>
-      <c r="H12" s="313"/>
-      <c r="I12" s="314"/>
-      <c r="J12" s="314"/>
-      <c r="K12" s="314"/>
-    </row>
     <row r="13" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A13" s="165"/>
-      <c r="B13" s="165"/>
-      <c r="C13" s="165"/>
-      <c r="D13" s="165"/>
-      <c r="E13" s="165"/>
-      <c r="F13" s="165"/>
-      <c r="G13" s="165"/>
-      <c r="H13" s="165"/>
-      <c r="I13" s="165"/>
-      <c r="J13" s="165"/>
-      <c r="K13" s="165"/>
+      <c r="A13" s="314"/>
+      <c r="B13" s="314"/>
+      <c r="C13" s="314"/>
+      <c r="D13" s="314"/>
+      <c r="E13" s="314"/>
+      <c r="F13" s="314"/>
+      <c r="G13" s="313" t="inlineStr">
+        <is>
+          <t>DIR-POL-06</t>
+        </is>
+      </c>
+      <c r="H13" s="313" t="inlineStr">
+        <is>
+          <t>Una dirección asociada a pedidos no se puede eliminar; el cliente puede registrar una nueva.</t>
+        </is>
+      </c>
+      <c r="I13" s="314"/>
+      <c r="J13" s="314"/>
+      <c r="K13" s="314"/>
     </row>
     <row r="14" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A14" s="165"/>
-      <c r="B14" s="165"/>
-      <c r="C14" s="165"/>
-      <c r="D14" s="165"/>
-      <c r="E14" s="165"/>
-      <c r="F14" s="165"/>
-      <c r="G14" s="165"/>
-      <c r="H14" s="165"/>
-      <c r="I14" s="165"/>
-      <c r="J14" s="165"/>
-      <c r="K14" s="165"/>
+      <c r="A14" s="313" t="str">
+        <f>ListadoObjetosDominio!B3</f>
+        <v>Cliente</v>
+      </c>
+      <c r="B14" s="313" t="inlineStr">
+        <is>
+          <t>Consultar direcciones</t>
+        </is>
+      </c>
+      <c r="C14" s="313" t="inlineStr">
+        <is>
+          <t>Listar las direcciones registradas por el cliente para seleccionarlas en el checkout.</t>
+        </is>
+      </c>
+      <c r="D14" s="313" t="str">
+        <f>ListadoObjetosDominio!B5</f>
+        <v>Dirección</v>
+      </c>
+      <c r="E14" s="313" t="inlineStr">
+        <is>
+          <t>idCliente</t>
+        </is>
+      </c>
+      <c r="F14" s="313" t="inlineStr">
+        <is>
+          <t>Selector de direcciones guardadas en el checkout y en el perfil del cliente.</t>
+        </is>
+      </c>
+      <c r="G14" s="313" t="inlineStr">
+        <is>
+          <t>DIR-POL-07</t>
+        </is>
+      </c>
+      <c r="H14" s="313" t="inlineStr">
+        <is>
+          <t>El cliente solo puede consultar sus propias direcciones; el administrador puede consultar todas.</t>
+        </is>
+      </c>
+      <c r="I14" s="313" t="s">
+        <v>180</v>
+      </c>
+      <c r="J14" s="313" t="inlineStr">
+        <is>
+          <t>Direcciones consultadas</t>
+        </is>
+      </c>
+      <c r="K14" s="313" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="65.25" customHeight="1">
+      <c r="A15" s="165"/>
+      <c r="B15" s="165"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="165"/>
+      <c r="E15" s="165"/>
+      <c r="F15" s="165"/>
+      <c r="G15" s="165"/>
+      <c r="H15" s="165"/>
+      <c r="I15" s="165"/>
+      <c r="J15" s="165"/>
+      <c r="K15" s="165"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F11:F12"/>
+  <mergeCells count="41">
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="F12:F13"/>
     <mergeCell ref="I7:I9"/>
-    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D12:D13"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="E12:E13"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B12:B13"/>
     <mergeCell ref="I5:I6"/>
-    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K12:K13"/>
     <mergeCell ref="J7:J9"/>
     <mergeCell ref="K7:K9"/>
     <mergeCell ref="G4:H4"/>
@@ -14405,18 +14516,25 @@
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="I12:I13"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="D5:D6"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="C7:C9"/>
     <mergeCell ref="D7:D9"/>
     <mergeCell ref="E7:E9"/>
     <mergeCell ref="F7:F9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:K11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de dominio'!A1" display="&lt;&lt; Ir al modelo de dominio" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
@@ -14556,47 +14674,51 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A11" s="313" t="s">
+      <c r="A11" s="246" t="s">
         <v>402</v>
       </c>
-      <c r="B11" s="313" t="s">
+      <c r="B11" s="246" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A12" s="313"/>
-      <c r="B12" s="313"/>
+      <c r="A12" s="246" t="inlineStr">
+        <is>
+          <t>DIR-POL-06</t>
+        </is>
+      </c>
+      <c r="B12" s="246" t="inlineStr">
+        <is>
+          <t>Una dirección asociada a pedidos no se puede eliminar; el cliente puede registrar una nueva.</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A13" s="165"/>
-      <c r="B13" s="165"/>
-      <c r="C13" s="165"/>
-      <c r="D13" s="165"/>
-      <c r="E13" s="165"/>
-      <c r="F13" s="165"/>
-      <c r="G13" s="165"/>
-      <c r="H13" s="165"/>
-      <c r="I13" s="165"/>
-      <c r="J13" s="165"/>
-      <c r="K13" s="165"/>
+      <c r="A13" s="246" t="inlineStr">
+        <is>
+          <t>DIR-POL-07</t>
+        </is>
+      </c>
+      <c r="B13" s="246" t="inlineStr">
+        <is>
+          <t>El cliente solo puede consultar sus propias direcciones; el administrador puede consultar todas.</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:13" ht="65.25" customHeight="1">
-      <c r="A14" s="165"/>
-      <c r="B14" s="165"/>
-      <c r="C14" s="165"/>
-      <c r="D14" s="165"/>
-      <c r="E14" s="165"/>
-      <c r="F14" s="165"/>
-      <c r="G14" s="165"/>
-      <c r="H14" s="165"/>
-      <c r="I14" s="165"/>
-      <c r="J14" s="165"/>
-      <c r="K14" s="165"/>
+      <c r="A14" s="246" t="inlineStr">
+        <is>
+          <t>DIR-POL-08</t>
+        </is>
+      </c>
+      <c r="B14" s="246" t="inlineStr">
+        <is>
+          <t>Una dirección asociada a pedidos en curso (Pendiente, Confirmado, Preparando o Enviado) no se puede modificar.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="A11:A12"/>
+  <mergeCells count="4">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B3:M3"/>

</xml_diff>